<commit_message>
Update standards data and related files
</commit_message>
<xml_diff>
--- a/input/metadata_v2.xlsx
+++ b/input/metadata_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/max/Documents/GitHub/HPLC_automatic_pre-processing/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaschwarz\repos\HPLC_automatic_pre-processing\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE822C8-DFD2-CB4E-817C-AA96446E5CB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5F9FEB-BF87-410B-9277-A49D45B5FC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1500" yWindow="1320" windowWidth="27640" windowHeight="16940" xr2:uid="{BB745C19-F00A-6F41-BD41-DCF17FCE42E9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{BB745C19-F00A-6F41-BD41-DCF17FCE42E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>temperature</t>
   </si>
@@ -82,28 +82,22 @@
     <t>Gua</t>
   </si>
   <si>
-    <t>20250407_ScADK_EbPPK_tmmcGAS</t>
-  </si>
-  <si>
     <t>MgCl2</t>
   </si>
   <si>
     <t>TrisHCL</t>
   </si>
   <si>
-    <t>20250619_ScADK_EaGK_EbPPK_tmmcGAS</t>
-  </si>
-  <si>
     <t>experiment_name</t>
   </si>
   <si>
-    <t>20241030 Ado ATP 1</t>
-  </si>
-  <si>
-    <t>20241030 Ado ATP 2</t>
-  </si>
-  <si>
-    <t>20241030 Ado ATP 3</t>
+    <t>20250617_EaGK_GTP_ATP_1</t>
+  </si>
+  <si>
+    <t>20250617_EaGK_GTP_ATP_2</t>
+  </si>
+  <si>
+    <t>20250617_EaGK_GTP_ATP_3</t>
   </si>
 </sst>
 </file>
@@ -159,9 +153,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -199,7 +193,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -305,7 +299,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -447,7 +441,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -455,16 +449,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DCE283C-6801-6B4B-AF83-67E669F4989C}">
-  <dimension ref="A1:R6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:R4"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
         <v>13</v>
@@ -476,51 +470,51 @@
         <v>1</v>
       </c>
       <c r="E1" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="F1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="K1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="P1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="Q1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="R1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -531,46 +525,43 @@
       <c r="D2">
         <v>8</v>
       </c>
-      <c r="E2">
-        <v>50000</v>
-      </c>
-      <c r="F2">
-        <v>5.6999999999999998E-4</v>
-      </c>
-      <c r="G2">
-        <v>1.06E-3</v>
-      </c>
       <c r="H2">
-        <v>7.2000000000000005E-4</v>
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="I2">
+        <v>5</v>
       </c>
       <c r="J2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L2">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M2">
         <v>0</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
       <c r="P2">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="Q2">
+        <v>50</v>
       </c>
       <c r="R2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -581,41 +572,41 @@
       <c r="D3">
         <v>8</v>
       </c>
-      <c r="E3">
-        <v>50000</v>
-      </c>
-      <c r="F3">
-        <v>5.6999999999999998E-4</v>
-      </c>
-      <c r="G3">
-        <v>7.2000000000000005E-4</v>
+      <c r="H3">
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I3">
-        <v>1.06E-3</v>
+        <v>5</v>
       </c>
       <c r="J3">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L3">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M3">
         <v>0</v>
       </c>
       <c r="N3">
-        <v>0.1</v>
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>5</v>
       </c>
       <c r="Q3">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="R3">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -628,140 +619,37 @@
       <c r="D4">
         <v>8</v>
       </c>
-      <c r="E4">
-        <v>50000</v>
-      </c>
-      <c r="F4">
-        <v>5.6999999999999998E-4</v>
-      </c>
-      <c r="G4">
-        <v>1.06E-3</v>
-      </c>
       <c r="H4">
-        <v>7.2000000000000005E-4</v>
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
       </c>
       <c r="J4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="L4">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>5</v>
+      </c>
+      <c r="Q4">
+        <v>50</v>
       </c>
       <c r="R4">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>21</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>37</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5">
-        <v>50000</v>
-      </c>
-      <c r="F5">
-        <v>5.6999999999999998E-4</v>
-      </c>
-      <c r="G5">
-        <v>1.06E-3</v>
-      </c>
-      <c r="H5">
-        <v>7.2000000000000005E-4</v>
-      </c>
-      <c r="J5">
-        <v>5</v>
-      </c>
-      <c r="K5">
-        <v>0.1</v>
-      </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>5</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="R5">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6">
-        <v>37</v>
-      </c>
-      <c r="D6">
-        <v>8</v>
-      </c>
-      <c r="E6">
-        <v>50000</v>
-      </c>
-      <c r="F6">
-        <v>5.6999999999999998E-4</v>
-      </c>
-      <c r="G6">
-        <v>1.06E-3</v>
-      </c>
-      <c r="H6">
-        <v>7.2000000000000005E-4</v>
-      </c>
-      <c r="J6">
-        <v>5</v>
-      </c>
-      <c r="K6">
-        <v>0.1</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>5</v>
-      </c>
-      <c r="O6">
-        <v>0</v>
-      </c>
-      <c r="P6">
-        <v>0</v>
-      </c>
-      <c r="R6">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
processing of the time samples is not working
</commit_message>
<xml_diff>
--- a/input/metadata_v2.xlsx
+++ b/input/metadata_v2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaschwarz\repos\HPLC_automatic_pre-processing\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B5F9FEB-BF87-410B-9277-A49D45B5FC5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEB0E268-17E0-4D1D-A095-2B9F18AE0D64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{BB745C19-F00A-6F41-BD41-DCF17FCE42E9}"/>
+    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="10360" xr2:uid="{BB745C19-F00A-6F41-BD41-DCF17FCE42E9}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>temperature</t>
   </si>
@@ -91,13 +91,16 @@
     <t>experiment_name</t>
   </si>
   <si>
-    <t>20250617_EaGK_GTP_ATP_1</t>
-  </si>
-  <si>
-    <t>20250617_EaGK_GTP_ATP_2</t>
-  </si>
-  <si>
-    <t>20250617_EaGK_GTP_ATP_3</t>
+    <t>PolyP</t>
+  </si>
+  <si>
+    <t>20241030 Ado ATP 1</t>
+  </si>
+  <si>
+    <t>20241030 Ado ATP 2</t>
+  </si>
+  <si>
+    <t>20241030 Ado ATP 3</t>
   </si>
 </sst>
 </file>
@@ -449,14 +452,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DCE283C-6801-6B4B-AF83-67E669F4989C}">
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="31.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -511,10 +514,13 @@
       <c r="R1" t="s">
         <v>15</v>
       </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -525,31 +531,13 @@
       <c r="D2">
         <v>8</v>
       </c>
-      <c r="H2">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="I2">
+      <c r="F2">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J2">
         <v>5</v>
       </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>5</v>
-      </c>
       <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
         <v>5</v>
       </c>
       <c r="Q2">
@@ -558,10 +546,13 @@
       <c r="R2">
         <v>10</v>
       </c>
+      <c r="S2">
+        <v>50</v>
+      </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -572,31 +563,13 @@
       <c r="D3">
         <v>8</v>
       </c>
-      <c r="H3">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="I3">
+      <c r="F3">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J3">
         <v>5</v>
       </c>
-      <c r="J3">
-        <v>0</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-      <c r="L3">
-        <v>5</v>
-      </c>
       <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>0</v>
-      </c>
-      <c r="P3">
         <v>5</v>
       </c>
       <c r="Q3">
@@ -605,10 +578,13 @@
       <c r="R3">
         <v>10</v>
       </c>
+      <c r="S3">
+        <v>50</v>
+      </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -619,31 +595,13 @@
       <c r="D4">
         <v>8</v>
       </c>
-      <c r="H4">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="I4">
+      <c r="F4">
+        <v>1.0000000000000001E-5</v>
+      </c>
+      <c r="J4">
         <v>5</v>
       </c>
-      <c r="J4">
-        <v>0</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-      <c r="L4">
-        <v>5</v>
-      </c>
       <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
         <v>5</v>
       </c>
       <c r="Q4">
@@ -651,9 +609,13 @@
       </c>
       <c r="R4">
         <v>10</v>
+      </c>
+      <c r="S4">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>